<commit_message>
feat: enhance onboarding steps and add floating social widget
- Updated Step2_FinancialDetails to improve button layout for mobile and desktop views.
- Refactored StepWrapper to adjust controls row styling and improve layout consistency.
- Introduced FloatingSocialWidget component for social media sharing with drag-and-drop functionality.
- Created socialLinks module to manage social media links and icons for the FloatingSocialWidget.
- Added CommunityDisclaimer component for legal notices in forums.
- Implemented GrantCardsPreview component to display government grants with loading and error states.
</commit_message>
<xml_diff>
--- a/government-data-extractor/output/government_schemes.xlsx
+++ b/government-data-extractor/output/government_schemes.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B635D7-CE89-4292-AD6A-E265D9C31F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Schemes" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Schemes" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="306">
   <si>
     <t>S.No</t>
   </si>
   <si>
+    <t>UI/UX Program Type</t>
+  </si>
+  <si>
+    <t>Scheme Name (official)</t>
+  </si>
+  <si>
     <t>UI/UX Short Description</t>
   </si>
   <si>
@@ -29,15 +31,9 @@
     <t>UI/UX Reference Link</t>
   </si>
   <si>
-    <t>UI/UX Program Type</t>
-  </si>
-  <si>
     <t>Scheme ID</t>
   </si>
   <si>
-    <t>Scheme Name (official)</t>
-  </si>
-  <si>
     <t>Acronym</t>
   </si>
   <si>
@@ -200,6 +196,12 @@
     <t>Catchy Line/Hook</t>
   </si>
   <si>
+    <t>Grant</t>
+  </si>
+  <si>
+    <t>First Home Owner (New Homes) Grant</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can receive a $10,000 grant when purchasing or building a home in NSW.</t>
   </si>
   <si>
@@ -209,15 +211,9 @@
     <t>https://www.revenue.nsw.gov.au/grants-schemes/first-home-owner-new-homes-grant</t>
   </si>
   <si>
-    <t>Grant</t>
-  </si>
-  <si>
     <t>nsw-first-home-owner-grant</t>
   </si>
   <si>
-    <t>First Home Owner (New Homes) Grant</t>
-  </si>
-  <si>
     <t>FHOG</t>
   </si>
   <si>
@@ -296,7 +292,7 @@
     <t>Via conveyancer/solicitor at settlement</t>
   </si>
   <si>
-    <t>2026-07-09</t>
+    <t>2026-07-17</t>
   </si>
   <si>
     <t>www.revenue.nsw.gov.au</t>
@@ -311,6 +307,9 @@
     <t>Get $10,000 towards your first home.</t>
   </si>
   <si>
+    <t>First Home Owner Grant</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can receive a $10,000 grant when purchasing or building a new home in VIC.</t>
   </si>
   <si>
@@ -323,9 +322,6 @@
     <t>vic-first-home-owner-grant</t>
   </si>
   <si>
-    <t>First Home Owner Grant</t>
-  </si>
-  <si>
     <t>State Revenue Office Victoria</t>
   </si>
   <si>
@@ -350,6 +346,9 @@
     <t>www.sro.vic.gov.au</t>
   </si>
   <si>
+    <t>First home owner grant</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can receive a $30,000 grant when purchasing or building a new home in QLD.</t>
   </si>
   <si>
@@ -362,9 +361,6 @@
     <t>qld-first-home-owner-grant</t>
   </si>
   <si>
-    <t>First home owner grant</t>
-  </si>
-  <si>
     <t>Queensland Revenue Office</t>
   </si>
   <si>
@@ -488,6 +484,9 @@
     <t>A cash boost for your first home.</t>
   </si>
   <si>
+    <t>HomeGrown Territory Grant</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can receive a $10,000 grant when purchasing or building a home in NT.</t>
   </si>
   <si>
@@ -500,9 +499,6 @@
     <t>nt-homegrown-territory-grant</t>
   </si>
   <si>
-    <t>HomeGrown Territory Grant</t>
-  </si>
-  <si>
     <t>HTG</t>
   </si>
   <si>
@@ -533,25 +529,25 @@
     <t>treasury.nt.gov.au</t>
   </si>
   <si>
+    <t>Scheme</t>
+  </si>
+  <si>
+    <t>Australian Government 5% Deposit Scheme</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can purchase a home with as little as a 5% deposit without paying Lenders Mortgage Insurance.</t>
   </si>
   <si>
-    <t>The First Home Guarantee allows eligible first home buyers to purchase a home with a minimum 5% deposit. The Australian Government guarantees part of the loan, helping eligible borrowers avoid paying Lenders Mortgage Insurance.</t>
-  </si>
-  <si>
-    <t>https://www.housingaustralia.gov.au/home-guarantee-scheme</t>
-  </si>
-  <si>
-    <t>Scheme</t>
-  </si>
-  <si>
-    <t>fed-first-home-guarantee</t>
-  </si>
-  <si>
-    <t>First Home Guarantee</t>
-  </si>
-  <si>
-    <t>FHBG</t>
+    <t>The Australian Government 5% Deposit Scheme allows eligible first home buyers to purchase a home with a minimum 5% deposit. The Australian Government guarantees part of the loan, helping eligible borrowers avoid paying Lenders Mortgage Insurance.</t>
+  </si>
+  <si>
+    <t>https://firsthomebuyers.gov.au/australian-government-5-percent-deposit-scheme</t>
+  </si>
+  <si>
+    <t>fed-5-percent-deposit-scheme</t>
+  </si>
+  <si>
+    <t>AGDS</t>
   </si>
   <si>
     <t>Guarantee</t>
@@ -566,6 +562,12 @@
     <t>All States &amp; Territories</t>
   </si>
   <si>
+    <t>Metro and regional (different caps may apply)</t>
+  </si>
+  <si>
+    <t>Use the Postcode Search Tool on the First Home Buyers website to check the price cap for the location you want to buy in.</t>
+  </si>
+  <si>
     <t>Government guarantee (avoids LMI)</t>
   </si>
   <si>
@@ -575,73 +577,64 @@
     <t>Buy with 5% deposit, government guarantees the balance to avoid LMI</t>
   </si>
   <si>
-    <t>New home; Apartment/Unit; Townhouse</t>
+    <t>$1,500,000</t>
+  </si>
+  <si>
+    <t>Varies by location: $1,500,000, $800,000, $950,000</t>
+  </si>
+  <si>
+    <t>Must not have owned property in Australia in the last 10 years</t>
   </si>
   <si>
     <t>Single parent</t>
   </si>
   <si>
-    <t>www.housingaustralia.gov.au</t>
-  </si>
-  <si>
-    <t>Please note that not all benefits, features, or entitlements listed may be applicable across all Schemes.</t>
+    <t>1 October 2025</t>
+  </si>
+  <si>
+    <t>1 July 2026</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>Statutory Declarations Act 1959; National Consumer Credit Protection Act 2009; Australian Citizenship Act 2007</t>
+  </si>
+  <si>
+    <t>firsthomebuyers.gov.au</t>
+  </si>
+  <si>
+    <t>Making a false or misleading statement is a serious offence •important: Part D is a Commonwealth Statutory Declaration.</t>
   </si>
   <si>
     <t>Low deposit, no LMI</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Buy with a low deposit — no Lenders Mortgage Insurance.</t>
   </si>
   <si>
-    <t>The Family Home Guarantee allows eligible first home buyers to purchase a home with a minimum 5% deposit. The Australian Government guarantees part of the loan, helping eligible borrowers avoid paying Lenders Mortgage Insurance.</t>
-  </si>
-  <si>
-    <t>fed-family-home-guarantee</t>
-  </si>
-  <si>
-    <t>Family Home Guarantee</t>
-  </si>
-  <si>
-    <t>FHG</t>
-  </si>
-  <si>
-    <t>The Regional First Home Buyer Guarantee allows eligible first home buyers to purchase a home with a minimum 5% deposit. The Australian Government guarantees part of the loan, helping eligible borrowers avoid paying Lenders Mortgage Insurance.</t>
-  </si>
-  <si>
-    <t>fed-regional-first-home-buyer-guarantee</t>
-  </si>
-  <si>
-    <t>Regional First Home Buyer Guarantee</t>
-  </si>
-  <si>
-    <t>RFHBG</t>
+    <t>Australian Government Help to Buy Scheme</t>
   </si>
   <si>
     <t>The government contributes toward the purchase price so eligible first home buyers can buy their first home with a smaller deposit.</t>
   </si>
   <si>
-    <t>Under the Help to Buy, the Australian Government contributes toward the purchase price of a home, reducing the deposit and loan an eligible first home buyer needs. Eligibility requirements are defined by Housing Australia.</t>
-  </si>
-  <si>
-    <t>https://www.housingaustralia.gov.au/home-guarantee-scheme/help-buy</t>
+    <t>Under the Australian Government Help to Buy Scheme, the Australian Government contributes toward the purchase price of a home, reducing the deposit and loan an eligible first home buyer needs. Applicants must satisfy residency, occupancy and income requirements defined by Housing Australia.</t>
+  </si>
+  <si>
+    <t>https://firsthomebuyers.gov.au/australian-government-help-buy-scheme</t>
   </si>
   <si>
     <t>fed-help-to-buy</t>
   </si>
   <si>
-    <t>Help to Buy</t>
-  </si>
-  <si>
     <t>HTB</t>
   </si>
   <si>
     <t>Shared Equity</t>
   </si>
   <si>
-    <t>Up to 5% equity contribution</t>
+    <t>Up to 2% equity contribution</t>
   </si>
   <si>
     <t>Equity share</t>
@@ -650,27 +643,51 @@
     <t>Government co-purchases a share of the property</t>
   </si>
   <si>
+    <t>Australian citizen</t>
+  </si>
+  <si>
+    <t>$103,000</t>
+  </si>
+  <si>
+    <t>$165,000</t>
+  </si>
+  <si>
+    <t>Taxable income</t>
+  </si>
+  <si>
+    <t>New home; Established home; Apartment/Unit; Townhouse</t>
+  </si>
+  <si>
+    <t>2%</t>
+  </si>
+  <si>
+    <t>You cannot apply directly to Housing Australia for Help to Buy.</t>
+  </si>
+  <si>
+    <t>10,000 places</t>
+  </si>
+  <si>
     <t>Shared equity</t>
   </si>
   <si>
     <t>Let the government co-buy your first home.</t>
   </si>
   <si>
+    <t>First Home Super Saver Scheme</t>
+  </si>
+  <si>
     <t>Eligible first home buyers can withdraw voluntary super contributions to help fund their first home deposit.</t>
   </si>
   <si>
-    <t>The First home super saver scheme lets eligible first home buyers withdraw eligible voluntary superannuation contributions to put toward their first home deposit. Eligibility requirements are defined by Australian Taxation Office.</t>
-  </si>
-  <si>
-    <t>https://www.ato.gov.au/individuals-and-families/super-for-individuals-and-families/super/withdrawing-and-using-your-super/early-access-to-super/first-home-super-saver-scheme</t>
+    <t>The First Home Super Saver Scheme lets eligible first home buyers withdraw eligible voluntary superannuation contributions to put toward their first home deposit. Applicants must satisfy ownership and residency requirements defined by Australian Taxation Office.</t>
+  </si>
+  <si>
+    <t>https://firsthomebuyers.gov.au/first-home-super-saver-scheme</t>
   </si>
   <si>
     <t>fed-first-home-super-saver</t>
   </si>
   <si>
-    <t>First home super saver scheme</t>
-  </si>
-  <si>
     <t>FHSSS</t>
   </si>
   <si>
@@ -680,7 +697,7 @@
     <t>Australian Taxation Office</t>
   </si>
   <si>
-    <t>Withdraw voluntary super contributions for a deposit</t>
+    <t>Withdraw up to $50,000 of voluntary super contributions</t>
   </si>
   <si>
     <t>Super withdrawal</t>
@@ -689,7 +706,10 @@
     <t>Withdraw eligible voluntary contributions plus associated earnings</t>
   </si>
   <si>
-    <t>www.ato.gov.au</t>
+    <t>New home; Established home; Vacant land</t>
+  </si>
+  <si>
+    <t>2025-10</t>
   </si>
   <si>
     <t>Super savings</t>
@@ -698,6 +718,9 @@
     <t>Supercharge your deposit through your super.</t>
   </si>
   <si>
+    <t>First Home Buyers Assistance Scheme</t>
+  </si>
+  <si>
     <t>Eligible first home buyers may pay reduced or no stamp duty when buying a home in NSW.</t>
   </si>
   <si>
@@ -710,9 +733,6 @@
     <t>nsw-first-home-buyers-assistance</t>
   </si>
   <si>
-    <t>First Home Buyers Assistance Scheme</t>
-  </si>
-  <si>
     <t>FHBAS</t>
   </si>
   <si>
@@ -761,6 +781,9 @@
     <t>Pay less (or no) stamp duty on your first home.</t>
   </si>
   <si>
+    <t>First home buyer duty exemption or concession</t>
+  </si>
+  <si>
     <t>Eligible first home buyers may pay reduced or no stamp duty when buying a home in VIC.</t>
   </si>
   <si>
@@ -773,9 +796,6 @@
     <t>vic-first-home-buyer-duty-exemption</t>
   </si>
   <si>
-    <t>First home buyer duty exemption or concession</t>
-  </si>
-  <si>
     <t>FBDEC</t>
   </si>
   <si>
@@ -788,12 +808,15 @@
     <t>New home; Established home; Off-the-plan; Vacant land</t>
   </si>
   <si>
-    <t>You are not eligible if you or your spouse or partner have already owned a home or other residential property in Australia.</t>
+    <t>You are not eligible if you, your spouse, or your partner have already owned a home or other residential property in Australia.</t>
   </si>
   <si>
     <t>Full exemption up to $750,000</t>
   </si>
   <si>
+    <t>First home concession</t>
+  </si>
+  <si>
     <t>Eligible first home buyers may pay reduced or no stamp duty when buying a home in QLD.</t>
   </si>
   <si>
@@ -806,9 +829,6 @@
     <t>qld-first-home-transfer-duty-concession</t>
   </si>
   <si>
-    <t>First home concession</t>
-  </si>
-  <si>
     <t>FC</t>
   </si>
   <si>
@@ -833,6 +853,9 @@
     <t>Rooming Accommodation Act 2008</t>
   </si>
   <si>
+    <t>First Home Owner Rate of Duty</t>
+  </si>
+  <si>
     <t>Eligible first home buyers may pay reduced or no stamp duty when buying an established home in WA.</t>
   </si>
   <si>
@@ -845,15 +868,9 @@
     <t>wa-first-home-owner-rate-of-duty</t>
   </si>
   <si>
-    <t>First Home Owner Rate of Duty</t>
-  </si>
-  <si>
     <t>FHOR</t>
   </si>
   <si>
-    <t>Australian citizen</t>
-  </si>
-  <si>
     <t>Varies by location: $800,000, $750,000, $1,000,000</t>
   </si>
   <si>
@@ -884,6 +901,9 @@
     <t>First Home Owner Grant Act 2000; Taxation Administration Act 2003; Duties Act 2008</t>
   </si>
   <si>
+    <t>Home Buyer Concession Scheme</t>
+  </si>
+  <si>
     <t>Eligible first home buyers may pay reduced or no stamp duty when buying a home in ACT.</t>
   </si>
   <si>
@@ -894,9 +914,6 @@
   </si>
   <si>
     <t>act-home-buyer-concession</t>
-  </si>
-  <si>
-    <t>Home Buyer Concession Scheme</t>
   </si>
   <si>
     <t>HBCS</t>
@@ -917,20 +934,18 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF111111"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1304,9 +1319,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BI16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1319,10 +1334,10 @@
     <col min="11" max="11" width="31" customWidth="1"/>
     <col min="12" max="13" width="60" customWidth="1"/>
     <col min="14" max="14" width="36" customWidth="1"/>
-    <col min="15" max="15" width="27" customWidth="1"/>
+    <col min="15" max="15" width="47" customWidth="1"/>
     <col min="16" max="16" width="60" customWidth="1"/>
     <col min="17" max="17" width="19" customWidth="1"/>
-    <col min="18" max="18" width="54" customWidth="1"/>
+    <col min="18" max="18" width="57" customWidth="1"/>
     <col min="19" max="19" width="21" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="33" customWidth="1"/>
@@ -1349,7 +1364,8 @@
     <col min="44" max="44" width="54" customWidth="1"/>
     <col min="45" max="45" width="22" customWidth="1"/>
     <col min="46" max="46" width="25" customWidth="1"/>
-    <col min="47" max="48" width="14" customWidth="1"/>
+    <col min="47" max="47" width="15" customWidth="1"/>
+    <col min="48" max="48" width="14" customWidth="1"/>
     <col min="49" max="49" width="19" customWidth="1"/>
     <col min="50" max="50" width="18" customWidth="1"/>
     <col min="51" max="51" width="36" customWidth="1"/>
@@ -1357,34 +1373,34 @@
     <col min="53" max="54" width="60" customWidth="1"/>
     <col min="55" max="55" width="42" customWidth="1"/>
     <col min="56" max="56" width="20" customWidth="1"/>
-    <col min="57" max="57" width="29" customWidth="1"/>
+    <col min="57" max="57" width="25" customWidth="1"/>
     <col min="58" max="58" width="60" customWidth="1"/>
     <col min="59" max="59" width="22" customWidth="1"/>
     <col min="60" max="60" width="18" customWidth="1"/>
     <col min="61" max="61" width="57" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" ht="30" customHeight="1" spans="1:61" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -1549,33 +1565,33 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:61" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>68</v>
@@ -1584,10 +1600,10 @@
         <v>69</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>70</v>
@@ -1599,7 +1615,7 @@
         <v>72</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>73</v>
@@ -1707,7 +1723,7 @@
         <v>71</v>
       </c>
       <c r="BA2" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="BB2" s="2" t="s">
         <v>91</v>
@@ -1734,33 +1750,33 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>67</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>68</v>
@@ -1769,10 +1785,10 @@
         <v>103</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>104</v>
@@ -1784,7 +1800,7 @@
         <v>71</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>73</v>
@@ -1892,7 +1908,7 @@
         <v>107</v>
       </c>
       <c r="BA3" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BB3" s="2" t="s">
         <v>108</v>
@@ -1919,33 +1935,33 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>67</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>68</v>
@@ -1954,10 +1970,10 @@
         <v>116</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>117</v>
@@ -1969,7 +1985,7 @@
         <v>71</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>119</v>
@@ -2077,7 +2093,7 @@
         <v>120</v>
       </c>
       <c r="BA4" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BB4" s="2" t="s">
         <v>71</v>
@@ -2104,15 +2120,15 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>124</v>
@@ -2130,7 +2146,7 @@
         <v>67</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>68</v>
@@ -2154,7 +2170,7 @@
         <v>71</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>73</v>
@@ -2289,15 +2305,15 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>133</v>
@@ -2315,7 +2331,7 @@
         <v>67</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>68</v>
@@ -2339,7 +2355,7 @@
         <v>71</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>139</v>
@@ -2474,15 +2490,15 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:61" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>148</v>
@@ -2500,7 +2516,7 @@
         <v>67</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>68</v>
@@ -2524,7 +2540,7 @@
         <v>71</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>71</v>
@@ -2659,33 +2675,33 @@
         <v>156</v>
       </c>
     </row>
-    <row r="8" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>160</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>162</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>163</v>
@@ -2694,10 +2710,10 @@
         <v>164</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>165</v>
@@ -2709,7 +2725,7 @@
         <v>71</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>73</v>
@@ -2817,7 +2833,7 @@
         <v>71</v>
       </c>
       <c r="BA8" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BB8" s="2" t="s">
         <v>71</v>
@@ -2844,27 +2860,27 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>178</v>
@@ -2879,28 +2895,28 @@
         <v>181</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>182</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>71</v>
+        <v>183</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>71</v>
+        <v>184</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>179</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="T9" s="2" t="s">
         <v>71</v>
@@ -2912,19 +2928,19 @@
         <v>71</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="X9" s="2" t="s">
         <v>77</v>
       </c>
       <c r="Y9" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>71</v>
+        <v>166</v>
       </c>
       <c r="AA9" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="AB9" s="2" t="s">
         <v>71</v>
@@ -2936,34 +2952,34 @@
         <v>71</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>71</v>
+        <v>188</v>
       </c>
       <c r="AF9" s="2" t="s">
-        <v>71</v>
+        <v>189</v>
       </c>
       <c r="AG9" s="2" t="s">
-        <v>186</v>
+        <v>81</v>
       </c>
       <c r="AH9" s="2" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="AI9" s="2" t="s">
         <v>130</v>
       </c>
       <c r="AJ9" s="2" t="s">
-        <v>71</v>
+        <v>190</v>
       </c>
       <c r="AK9" s="2" t="s">
         <v>77</v>
       </c>
       <c r="AL9" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AM9" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="AN9" s="2" t="s">
-        <v>71</v>
+        <v>142</v>
       </c>
       <c r="AO9" s="2" t="s">
         <v>71</v>
@@ -2990,72 +3006,72 @@
         <v>87</v>
       </c>
       <c r="AW9" s="2" t="s">
-        <v>71</v>
+        <v>192</v>
       </c>
       <c r="AX9" s="2" t="s">
-        <v>71</v>
+        <v>193</v>
       </c>
       <c r="AY9" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AZ9" s="2" t="s">
-        <v>71</v>
+        <v>194</v>
       </c>
       <c r="BA9" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BB9" s="2" t="s">
-        <v>71</v>
+        <v>195</v>
       </c>
       <c r="BC9" s="2" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
       <c r="BD9" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE9" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="BF9" s="2" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="BG9" s="2" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="BH9" s="2" t="s">
-        <v>191</v>
+        <v>96</v>
       </c>
       <c r="BI9" s="2" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>180</v>
@@ -3064,10 +3080,10 @@
         <v>181</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>172</v>
+        <v>201</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>182</v>
@@ -3079,13 +3095,13 @@
         <v>71</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="T10" s="2" t="s">
         <v>71</v>
@@ -3097,28 +3113,28 @@
         <v>71</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="X10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="Y10" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="Y10" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="Z10" s="2" t="s">
-        <v>71</v>
+        <v>210</v>
       </c>
       <c r="AA10" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="AB10" s="2" t="s">
-        <v>71</v>
+        <v>211</v>
       </c>
       <c r="AC10" s="2" t="s">
-        <v>71</v>
+        <v>212</v>
       </c>
       <c r="AD10" s="2" t="s">
-        <v>71</v>
+        <v>213</v>
       </c>
       <c r="AE10" s="2" t="s">
         <v>71</v>
@@ -3127,13 +3143,13 @@
         <v>71</v>
       </c>
       <c r="AG10" s="2" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="AH10" s="2" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="AI10" s="2" t="s">
-        <v>130</v>
+        <v>215</v>
       </c>
       <c r="AJ10" s="2" t="s">
         <v>71</v>
@@ -3145,13 +3161,13 @@
         <v>71</v>
       </c>
       <c r="AM10" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="AN10" s="2" t="s">
-        <v>71</v>
+        <v>131</v>
       </c>
       <c r="AO10" s="2" t="s">
-        <v>71</v>
+        <v>216</v>
       </c>
       <c r="AP10" s="2" t="s">
         <v>71</v>
@@ -3169,7 +3185,7 @@
         <v>71</v>
       </c>
       <c r="AU10" s="2" t="s">
-        <v>71</v>
+        <v>217</v>
       </c>
       <c r="AV10" s="2" t="s">
         <v>87</v>
@@ -3187,72 +3203,72 @@
         <v>71</v>
       </c>
       <c r="BA10" s="2" t="s">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="BB10" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BC10" s="2" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
       <c r="BD10" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE10" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="BF10" s="2" t="s">
-        <v>189</v>
+        <v>71</v>
       </c>
       <c r="BG10" s="2" t="s">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="BH10" s="2" t="s">
-        <v>191</v>
+        <v>96</v>
       </c>
       <c r="BI10" s="2" t="s">
-        <v>192</v>
+        <v>219</v>
       </c>
     </row>
-    <row r="11" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>172</v>
+        <v>221</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>174</v>
+        <v>223</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>180</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>181</v>
+        <v>227</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>172</v>
+        <v>221</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>197</v>
+        <v>222</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>182</v>
@@ -3264,13 +3280,13 @@
         <v>71</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>183</v>
+        <v>228</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>184</v>
+        <v>229</v>
       </c>
       <c r="T11" s="2" t="s">
         <v>71</v>
@@ -3282,19 +3298,19 @@
         <v>71</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>185</v>
+        <v>230</v>
       </c>
       <c r="X11" s="2" t="s">
         <v>77</v>
       </c>
       <c r="Y11" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>71</v>
+        <v>210</v>
       </c>
       <c r="AA11" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="AB11" s="2" t="s">
         <v>71</v>
@@ -3312,25 +3328,25 @@
         <v>71</v>
       </c>
       <c r="AG11" s="2" t="s">
-        <v>186</v>
+        <v>231</v>
       </c>
       <c r="AH11" s="2" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="AI11" s="2" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="AJ11" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="AK11" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="AL11" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AM11" s="2" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
       <c r="AN11" s="2" t="s">
         <v>71</v>
@@ -3369,93 +3385,93 @@
         <v>71</v>
       </c>
       <c r="AZ11" s="2" t="s">
-        <v>71</v>
+        <v>232</v>
       </c>
       <c r="BA11" s="2" t="s">
-        <v>174</v>
+        <v>223</v>
       </c>
       <c r="BB11" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BC11" s="2" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="BD11" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE11" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="BF11" s="2" t="s">
-        <v>189</v>
+        <v>71</v>
       </c>
       <c r="BG11" s="2" t="s">
-        <v>190</v>
+        <v>233</v>
       </c>
       <c r="BH11" s="2" t="s">
-        <v>191</v>
+        <v>96</v>
       </c>
       <c r="BI11" s="2" t="s">
-        <v>192</v>
+        <v>234</v>
       </c>
     </row>
-    <row r="12" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>207</v>
+        <v>241</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>180</v>
+        <v>68</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>181</v>
+        <v>69</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>182</v>
+        <v>70</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>71</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>71</v>
+        <v>242</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>207</v>
+        <v>241</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>208</v>
+        <v>243</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>209</v>
+        <v>244</v>
       </c>
       <c r="T12" s="2" t="s">
         <v>71</v>
@@ -3467,19 +3483,19 @@
         <v>71</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>210</v>
+        <v>245</v>
       </c>
       <c r="X12" s="2" t="s">
         <v>77</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="AB12" s="2" t="s">
         <v>71</v>
@@ -3497,40 +3513,40 @@
         <v>71</v>
       </c>
       <c r="AG12" s="2" t="s">
-        <v>186</v>
+        <v>246</v>
       </c>
       <c r="AH12" s="2" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="AI12" s="2" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="AJ12" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="AK12" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="AL12" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AM12" s="2" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
       <c r="AN12" s="2" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="AO12" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AP12" s="2" t="s">
-        <v>71</v>
+        <v>247</v>
       </c>
       <c r="AQ12" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AR12" s="2" t="s">
-        <v>71</v>
+        <v>248</v>
       </c>
       <c r="AS12" s="2" t="s">
         <v>71</v>
@@ -3545,87 +3561,87 @@
         <v>87</v>
       </c>
       <c r="AW12" s="2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="AX12" s="2" t="s">
-        <v>71</v>
+        <v>249</v>
       </c>
       <c r="AY12" s="2" t="s">
-        <v>71</v>
+        <v>250</v>
       </c>
       <c r="AZ12" s="2" t="s">
-        <v>71</v>
+        <v>251</v>
       </c>
       <c r="BA12" s="2" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="BB12" s="2" t="s">
-        <v>71</v>
+        <v>252</v>
       </c>
       <c r="BC12" s="2" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="BD12" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE12" s="2" t="s">
-        <v>188</v>
+        <v>94</v>
       </c>
       <c r="BF12" s="2" t="s">
-        <v>189</v>
+        <v>71</v>
       </c>
       <c r="BG12" s="2" t="s">
-        <v>211</v>
+        <v>253</v>
       </c>
       <c r="BH12" s="2" t="s">
-        <v>96</v>
+        <v>254</v>
       </c>
       <c r="BI12" s="2" t="s">
-        <v>212</v>
+        <v>255</v>
       </c>
     </row>
-    <row r="13" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>217</v>
+        <v>256</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>213</v>
+        <v>257</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>214</v>
+        <v>258</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>218</v>
+        <v>261</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>219</v>
+        <v>262</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>180</v>
+        <v>68</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>220</v>
+        <v>103</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>213</v>
+        <v>257</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>214</v>
+        <v>258</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>182</v>
+        <v>104</v>
       </c>
       <c r="O13" s="2" t="s">
         <v>71</v>
@@ -3634,13 +3650,13 @@
         <v>71</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>219</v>
+        <v>262</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="T13" s="2" t="s">
         <v>71</v>
@@ -3652,19 +3668,19 @@
         <v>71</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="X13" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="Y13" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>71</v>
+        <v>166</v>
       </c>
       <c r="AA13" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="AB13" s="2" t="s">
         <v>71</v>
@@ -3676,22 +3692,22 @@
         <v>71</v>
       </c>
       <c r="AE13" s="2" t="s">
-        <v>71</v>
+        <v>263</v>
       </c>
       <c r="AF13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AG13" s="2" t="s">
-        <v>71</v>
+        <v>264</v>
       </c>
       <c r="AH13" s="2" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="AI13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AJ13" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="AK13" s="2" t="s">
         <v>71</v>
@@ -3700,22 +3716,22 @@
         <v>71</v>
       </c>
       <c r="AM13" s="2" t="s">
-        <v>71</v>
+        <v>141</v>
       </c>
       <c r="AN13" s="2" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="AO13" s="2" t="s">
-        <v>71</v>
+        <v>265</v>
       </c>
       <c r="AP13" s="2" t="s">
-        <v>71</v>
+        <v>263</v>
       </c>
       <c r="AQ13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AR13" s="2" t="s">
-        <v>71</v>
+        <v>266</v>
       </c>
       <c r="AS13" s="2" t="s">
         <v>71</v>
@@ -3730,102 +3746,102 @@
         <v>87</v>
       </c>
       <c r="AW13" s="2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="AX13" s="2" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="AY13" s="2" t="s">
-        <v>71</v>
+        <v>250</v>
       </c>
       <c r="AZ13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BA13" s="2" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="BB13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BC13" s="2" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="BD13" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE13" s="2" t="s">
-        <v>224</v>
+        <v>110</v>
       </c>
       <c r="BF13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BG13" s="2" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="BH13" s="2" t="s">
-        <v>96</v>
+        <v>254</v>
       </c>
       <c r="BI13" s="2" t="s">
-        <v>226</v>
+        <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>231</v>
+        <v>267</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>227</v>
+        <v>268</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>228</v>
+        <v>269</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>229</v>
+        <v>270</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>232</v>
+        <v>272</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>68</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>227</v>
+        <v>268</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>228</v>
+        <v>269</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>70</v>
+        <v>117</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>234</v>
+        <v>71</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="T14" s="2" t="s">
         <v>71</v>
@@ -3837,7 +3853,7 @@
         <v>71</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="X14" s="2" t="s">
         <v>77</v>
@@ -3846,7 +3862,7 @@
         <v>77</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>78</v>
+        <v>166</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>79</v>
@@ -3867,7 +3883,7 @@
         <v>71</v>
       </c>
       <c r="AG14" s="2" t="s">
-        <v>238</v>
+        <v>273</v>
       </c>
       <c r="AH14" s="2" t="s">
         <v>82</v>
@@ -3885,22 +3901,22 @@
         <v>71</v>
       </c>
       <c r="AM14" s="2" t="s">
-        <v>141</v>
+        <v>84</v>
       </c>
       <c r="AN14" s="2" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="AO14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AP14" s="2" t="s">
-        <v>239</v>
+        <v>274</v>
       </c>
       <c r="AQ14" s="2" t="s">
-        <v>71</v>
+        <v>275</v>
       </c>
       <c r="AR14" s="2" t="s">
-        <v>240</v>
+        <v>276</v>
       </c>
       <c r="AS14" s="2" t="s">
         <v>71</v>
@@ -3915,87 +3931,87 @@
         <v>87</v>
       </c>
       <c r="AW14" s="2" t="s">
-        <v>89</v>
+        <v>277</v>
       </c>
       <c r="AX14" s="2" t="s">
-        <v>241</v>
+        <v>277</v>
       </c>
       <c r="AY14" s="2" t="s">
-        <v>242</v>
+        <v>278</v>
       </c>
       <c r="AZ14" s="2" t="s">
-        <v>243</v>
+        <v>71</v>
       </c>
       <c r="BA14" s="2" t="s">
-        <v>229</v>
+        <v>270</v>
       </c>
       <c r="BB14" s="2" t="s">
-        <v>244</v>
+        <v>279</v>
       </c>
       <c r="BC14" s="2" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="BD14" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE14" s="2" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="BF14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BG14" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="BH14" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="BI14" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
-    <row r="15" spans="1:61" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>252</v>
+        <v>280</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>250</v>
+        <v>283</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>251</v>
+        <v>284</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>253</v>
+        <v>285</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>68</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>71</v>
@@ -4004,13 +4020,13 @@
         <v>71</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="T15" s="2" t="s">
         <v>71</v>
@@ -4022,19 +4038,19 @@
         <v>71</v>
       </c>
       <c r="W15" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="X15" s="2" t="s">
         <v>77</v>
       </c>
       <c r="Y15" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="Z15" s="2" t="s">
-        <v>166</v>
+        <v>210</v>
       </c>
       <c r="AA15" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="AB15" s="2" t="s">
         <v>71</v>
@@ -4046,22 +4062,22 @@
         <v>71</v>
       </c>
       <c r="AE15" s="2" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="AF15" s="2" t="s">
-        <v>71</v>
+        <v>286</v>
       </c>
       <c r="AG15" s="2" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="AH15" s="2" t="s">
-        <v>82</v>
+        <v>288</v>
       </c>
       <c r="AI15" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AJ15" s="2" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="AK15" s="2" t="s">
         <v>71</v>
@@ -4073,19 +4089,19 @@
         <v>141</v>
       </c>
       <c r="AN15" s="2" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="AO15" s="2" t="s">
-        <v>257</v>
+        <v>71</v>
       </c>
       <c r="AP15" s="2" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="AQ15" s="2" t="s">
-        <v>71</v>
+        <v>289</v>
       </c>
       <c r="AR15" s="2" t="s">
-        <v>258</v>
+        <v>290</v>
       </c>
       <c r="AS15" s="2" t="s">
         <v>71</v>
@@ -4100,22 +4116,22 @@
         <v>87</v>
       </c>
       <c r="AW15" s="2" t="s">
-        <v>89</v>
+        <v>291</v>
       </c>
       <c r="AX15" s="2" t="s">
-        <v>89</v>
+        <v>292</v>
       </c>
       <c r="AY15" s="2" t="s">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="AZ15" s="2" t="s">
-        <v>71</v>
+        <v>294</v>
       </c>
       <c r="BA15" s="2" t="s">
-        <v>250</v>
+        <v>283</v>
       </c>
       <c r="BB15" s="2" t="s">
-        <v>71</v>
+        <v>295</v>
       </c>
       <c r="BC15" s="2" t="s">
         <v>121</v>
@@ -4124,63 +4140,63 @@
         <v>93</v>
       </c>
       <c r="BE15" s="2" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="BF15" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BG15" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="BH15" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="BI15" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:61" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>263</v>
+        <v>296</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>259</v>
+        <v>297</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>260</v>
+        <v>298</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>261</v>
+        <v>299</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>262</v>
+        <v>300</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>264</v>
+        <v>301</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>68</v>
+        <v>163</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>116</v>
+        <v>302</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>259</v>
+        <v>297</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>260</v>
+        <v>298</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>117</v>
+        <v>303</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>71</v>
@@ -4189,13 +4205,13 @@
         <v>71</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="T16" s="2" t="s">
         <v>71</v>
@@ -4207,19 +4223,19 @@
         <v>71</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="X16" s="2" t="s">
         <v>77</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="Z16" s="2" t="s">
-        <v>166</v>
+        <v>71</v>
       </c>
       <c r="AA16" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="AB16" s="2" t="s">
         <v>71</v>
@@ -4237,16 +4253,16 @@
         <v>71</v>
       </c>
       <c r="AG16" s="2" t="s">
-        <v>265</v>
+        <v>71</v>
       </c>
       <c r="AH16" s="2" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="AI16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AJ16" s="2" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="AK16" s="2" t="s">
         <v>71</v>
@@ -4255,22 +4271,22 @@
         <v>71</v>
       </c>
       <c r="AM16" s="2" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="AN16" s="2" t="s">
-        <v>131</v>
+        <v>71</v>
       </c>
       <c r="AO16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="AP16" s="2" t="s">
-        <v>266</v>
+        <v>71</v>
       </c>
       <c r="AQ16" s="2" t="s">
-        <v>267</v>
+        <v>71</v>
       </c>
       <c r="AR16" s="2" t="s">
-        <v>268</v>
+        <v>71</v>
       </c>
       <c r="AS16" s="2" t="s">
         <v>71</v>
@@ -4285,417 +4301,47 @@
         <v>87</v>
       </c>
       <c r="AW16" s="2" t="s">
-        <v>269</v>
+        <v>71</v>
       </c>
       <c r="AX16" s="2" t="s">
-        <v>269</v>
+        <v>304</v>
       </c>
       <c r="AY16" s="2" t="s">
-        <v>270</v>
+        <v>304</v>
       </c>
       <c r="AZ16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BA16" s="2" t="s">
-        <v>261</v>
+        <v>299</v>
       </c>
       <c r="BB16" s="2" t="s">
-        <v>271</v>
+        <v>71</v>
       </c>
       <c r="BC16" s="2" t="s">
-        <v>121</v>
+        <v>71</v>
       </c>
       <c r="BD16" s="2" t="s">
         <v>93</v>
       </c>
       <c r="BE16" s="2" t="s">
-        <v>122</v>
+        <v>305</v>
       </c>
       <c r="BF16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="BG16" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="BH16" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="BI16" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="17" spans="1:61" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="A17" s="2">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="P17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q17" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="S17" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="T17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="U17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="V17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="W17" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="X17" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="Z17" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="AA17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AB17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AC17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AD17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE17" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="AF17" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="AG17" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="AH17" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="AI17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AK17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AM17" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AN17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AO17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AP17" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="AQ17" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="AR17" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="AS17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AT17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AU17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AV17" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AW17" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="AX17" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="AY17" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="AZ17" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="BA17" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="BB17" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="BC17" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="BD17" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="BE17" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BF17" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BG17" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="BH17" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="BI17" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="18" spans="1:61" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="P18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="R18" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="S18" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="T18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="U18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="V18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="W18" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="X18" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="Z18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AB18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AC18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AD18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AF18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AG18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AI18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AK18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AM18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AN18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AO18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AP18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AQ18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AR18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AS18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AT18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AU18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AV18" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AW18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AX18" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="AY18" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="AZ18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BA18" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="BB18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BC18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BD18" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="BE18" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="BF18" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BG18" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="BH18" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="BI18" s="2" t="s">
-        <v>247</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>